<commit_message>
Vídeo 1 aula 2
</commit_message>
<xml_diff>
--- a/Analise_de_dados_e_IA_Nivelamento/Semana_01/Excel/Domine_o_editor_de_planilhas/src/Meteora Ecommerce_Aula1.xlsx
+++ b/Analise_de_dados_e_IA_Nivelamento/Semana_01/Excel/Domine_o_editor_de_planilhas/src/Meteora Ecommerce_Aula1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://officeresolve-my.sharepoint.com/personal/r_sabino_officeresolve_com_br/Documents/Alura-Ciência de Dados/03.01 - Novas Formações Excel/Formação Excel/3195 - Excel 1 - Domine o Editor de planilhas/Materiais do Curso/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thierry-G15\Documents\Estudos\Alura\Santander-Imersao-Digital\Analise_de_dados_e_IA_Nivelamento\Semana_01\Excel\Domine_o_editor_de_planilhas\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="8_{0D071335-E186-43B8-A2BC-FF91FCFBAFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{653020B6-5AB9-4AB9-9CCB-FC0BB8A301C6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6E1EF72-89F3-46D6-A1F5-8D5499707352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="16">
   <si>
     <t>Produtos</t>
   </si>
@@ -84,21 +84,6 @@
   </si>
   <si>
     <t>Camiseta Lisa</t>
-  </si>
-  <si>
-    <t>Categoria</t>
-  </si>
-  <si>
-    <t>Preço Unitário</t>
-  </si>
-  <si>
-    <t>Vestuário</t>
-  </si>
-  <si>
-    <t>Acessórios</t>
-  </si>
-  <si>
-    <t>Calçado</t>
   </si>
 </sst>
 </file>
@@ -464,307 +449,181 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7162DC3F-8DD7-4F1A-A109-A490D58F15DD}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2">
-        <v>25.9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3">
-        <v>29.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4">
-        <v>32.9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5">
-        <v>399.9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6">
-        <v>249.9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7">
-        <v>259.89999999999998</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8">
-        <v>299.89999999999998</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9">
-        <v>85.9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10">
-        <v>89.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11">
-        <v>92.9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12">
-        <v>149.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13">
-        <v>65.900000000000006</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14">
-        <v>69.900000000000006</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15">
-        <v>70.900000000000006</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="1">
         <v>36</v>
       </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16">
-        <v>199.9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="1">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
-        <v>20</v>
-      </c>
-      <c r="D17">
-        <v>249.9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>10</v>
       </c>
       <c r="B18" s="1">
         <v>38</v>
       </c>
-      <c r="C18" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18">
-        <v>259.89999999999998</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19">
-        <v>259.89999999999998</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C20" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20">
-        <v>39.9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="C21" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21">
-        <v>49.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>